<commit_message>
Finalize native Excel chart output
</commit_message>
<xml_diff>
--- a/templates/attributed-growth-by-segment-template/attributed_growth_by_segment_blank_template.xlsx
+++ b/templates/attributed-growth-by-segment-template/attributed_growth_by_segment_blank_template.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Attributed Growth" sheetId="1" r:id="rId1"/>
-    <sheet name="_Native Chart" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Attributed Growth'!$A$1:$N$32</definedName>
@@ -18,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
   <si>
     <t>1. Attributed Growth by Segment Template</t>
   </si>
@@ -65,9 +64,6 @@
     <t>CS + Ins.</t>
   </si>
   <si>
-    <t>Attributed</t>
-  </si>
-  <si>
     <t>RBC</t>
   </si>
   <si>
@@ -83,10 +79,67 @@
     <t>National Bank</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>TD</t>
+  </si>
+  <si>
+    <t>CB Chart Value</t>
+  </si>
+  <si>
+    <t>IB Chart Value</t>
+  </si>
+  <si>
+    <t>CM Chart Value</t>
+  </si>
+  <si>
+    <t>WM Chart Value</t>
+  </si>
+  <si>
+    <t>CS + Ins. Chart Value</t>
+  </si>
+  <si>
+    <t>CB Label X</t>
+  </si>
+  <si>
+    <t>CB Label Y</t>
+  </si>
+  <si>
+    <t>CB Label</t>
+  </si>
+  <si>
+    <t>IB Label X</t>
+  </si>
+  <si>
+    <t>IB Label Y</t>
+  </si>
+  <si>
+    <t>IB Label</t>
+  </si>
+  <si>
+    <t>CM Label X</t>
+  </si>
+  <si>
+    <t>CM Label Y</t>
+  </si>
+  <si>
+    <t>CM Label</t>
+  </si>
+  <si>
+    <t>WM Label X</t>
+  </si>
+  <si>
+    <t>WM Label Y</t>
+  </si>
+  <si>
+    <t>WM Label</t>
+  </si>
+  <si>
+    <t>CS + Ins. Label X</t>
+  </si>
+  <si>
+    <t>CS + Ins. Label Y</t>
+  </si>
+  <si>
+    <t>CS + Ins. Label</t>
   </si>
 </sst>
 </file>
@@ -264,7 +317,17 @@
   <c:chart>
     <c:autoTitleDeleted val="1"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.061350000000000002"/>
+          <c:y val="0.070000000000000007"/>
+          <c:w val="0.88339999999999996"/>
+          <c:h val="0.92000000000000004"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="stacked"/>
@@ -288,29 +351,10 @@
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
+                <a:srgbClr val="40484A"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
-            <c:txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="ctr"/>
-            <c:showVal val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
@@ -339,27 +383,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Attributed Growth'!$S$5:$S$10</c:f>
+              <c:f>'Attributed Growth'!$Y$5:$Y$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -385,29 +429,10 @@
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
+                <a:srgbClr val="001A52"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
-            <c:txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="ctr"/>
-            <c:showVal val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
@@ -436,27 +461,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Attributed Growth'!$T$5:$T$10</c:f>
+              <c:f>'Attributed Growth'!$Z$5:$Z$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -482,29 +507,10 @@
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
+                <a:srgbClr val="2D5967"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
-            <c:txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="FFFFFF"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="ctr"/>
-            <c:showVal val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
@@ -533,27 +539,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Attributed Growth'!$U$5:$U$10</c:f>
+              <c:f>'Attributed Growth'!$AA$5:$AA$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -579,29 +585,10 @@
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
+                <a:srgbClr val="F28C00"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
-            <c:txPr>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1200" baseline="0">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="ctr"/>
-            <c:showVal val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
@@ -630,27 +617,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Attributed Growth'!$V$5:$V$10</c:f>
+              <c:f>'Attributed Growth'!$AB$5:$AB$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -676,18 +663,195 @@
             </a:solidFill>
             <a:ln>
               <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
+                <a:srgbClr val="000000"/>
               </a:solidFill>
             </a:ln>
           </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>RBC</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>BMO</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Scotia</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>CIBC</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>National Bank</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>TD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AC$5:$AC$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="70"/>
+        <c:overlap val="100"/>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
           <c:dLbls>
-            <c:numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$5</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$6</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$7</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$8</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$9</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AH$10</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="40484A"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="40484A"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
             <c:txPr>
               <a:bodyPr/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1200" baseline="0">
+                  <a:defRPr sz="1200" b="1" baseline="0">
                     <a:solidFill>
                       <a:srgbClr val="FFFFFF"/>
                     </a:solidFill>
@@ -697,78 +861,835 @@
               </a:p>
             </c:txPr>
             <c:dLblPos val="ctr"/>
-            <c:showVal val="1"/>
           </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'Attributed Growth'!$P$5:$P$10</c:f>
-              <c:strCache>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>RBC</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>BMO</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Scotia</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>CIBC</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>National Bank</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>TD</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
+          <c:xVal>
             <c:numRef>
-              <c:f>'Attributed Growth'!$W$5:$W$10</c:f>
+              <c:f>'Attributed Growth'!$AF$5:$AF$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2.9</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>3.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>4.9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>5.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AG$5:$AG$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.05</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
         </c:ser>
-        <c:gapWidth val="70"/>
-        <c:overlap val="100"/>
-        <c:axId val="50010001"/>
-        <c:axId val="50010002"/>
-      </c:barChart>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$5</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$6</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$7</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$8</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$9</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AK$10</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="001A52"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="001A52"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AI$5:$AI$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AJ$5:$AJ$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.15000000000000002</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$5</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$6</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$7</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$8</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$9</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AN$10</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2D5967"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2D5967"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AL$5:$AL$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AM$5:$AM$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$5</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$6</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$7</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$8</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$9</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AQ$10</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F28C00"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="F28C00"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AO$5:$AO$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.08</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.08</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4.08</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.08</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.08</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AP$5:$AP$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.35000000000000003</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="9"/>
+          <c:order val="9"/>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$5</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$6</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$7</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$8</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$9</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="5"/>
+              <c:layout/>
+              <c:tx>
+                <c:strRef>
+                  <c:f>'Attributed Growth'!$AT$10</c:f>
+                  <c:strCache>
+                    <c:ptCount val="1"/>
+                    <c:pt idx="0">
+                      <c:v>0%</c:v>
+                    </c:pt>
+                  </c:strCache>
+                </c:strRef>
+              </c:tx>
+              <c:dLblPos val="ctr"/>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1200" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="FFFFFF"/>
+                    </a:solidFill>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="ctr"/>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AR$5:$AR$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.92</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.92</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.92</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.92</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.92</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.92</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Attributed Growth'!$AS$5:$AS$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.45</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.45</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:axId val="60010001"/>
+        <c:axId val="60010002"/>
+      </c:scatterChart>
       <c:catAx>
         <c:axId val="50010001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:delete val="1"/>
         <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
-          <a:ln>
-            <a:noFill/>
+          <a:ln w="15875">
+            <a:solidFill>
+              <a:srgbClr val="8C8C8C"/>
+            </a:solidFill>
           </a:ln>
         </c:spPr>
         <c:txPr>
@@ -776,7 +1697,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr baseline="0">
+              <a:defRPr sz="100" baseline="0">
                 <a:solidFill>
                   <a:srgbClr val="FFFFFF"/>
                 </a:solidFill>
@@ -812,6 +1733,74 @@
         <c:crossBetween val="between"/>
         <c:majorUnit val="5"/>
       </c:valAx>
+      <c:valAx>
+        <c:axId val="60010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="100" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="60010001"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="5"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="60010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="none"/>
+        <c:spPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="100" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="60010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
       <c:spPr>
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
@@ -1068,72 +2057,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="TextBox 7"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="628650" y="5610225"/>
-          <a:ext cx="9677400" cy="19050"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="8C8C8C"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" b="1">
-            <a:solidFill>
-              <a:srgbClr val="000000"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1143,13 +2066,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="8" name="Chart 7"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1158,7 +2081,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1168,9 +2091,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AttributedGrowthBySegmentSource" displayName="AttributedGrowthBySegmentSource" ref="P4:X10" totalsRowShown="0">
-  <autoFilter ref="P4:X10"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AttributedGrowthBySegmentSource" displayName="AttributedGrowthBySegmentSource" ref="P4:W10" totalsRowShown="0">
+  <autoFilter ref="P4:W10"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Bank"/>
     <tableColumn id="2" name="Absolute Growth ($BN)"/>
     <tableColumn id="3" name="Reported YoY Growth"/>
@@ -1179,7 +2102,6 @@
     <tableColumn id="6" name="CM"/>
     <tableColumn id="7" name="WM"/>
     <tableColumn id="8" name="CS + Ins."/>
-    <tableColumn id="9" name="Attributed"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1473,7 +2395,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y32"/>
+  <dimension ref="A1:AT32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1483,10 +2405,12 @@
     <col min="17" max="17" width="16.85546875" customWidth="1"/>
     <col min="18" max="18" width="15" customWidth="1"/>
     <col min="19" max="22" width="10" customWidth="1"/>
-    <col min="23" max="25" width="12.140625" customWidth="1"/>
+    <col min="23" max="24" width="12.140625" customWidth="1"/>
+    <col min="25" max="29" width="0" hidden="1" customWidth="1"/>
+    <col min="32" max="46" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="27" customHeight="1">
+    <row r="1" spans="1:46" ht="27" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1515,7 +2439,7 @@
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
     </row>
-    <row r="2" spans="1:25" ht="18" customHeight="1">
+    <row r="2" spans="1:46" ht="18" customHeight="1">
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1538,8 +2462,8 @@
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
     </row>
-    <row r="3" spans="1:25" ht="7.5" customHeight="1"/>
-    <row r="4" spans="1:25">
+    <row r="3" spans="1:46" ht="7.5" customHeight="1"/>
+    <row r="4" spans="1:46">
       <c r="C4" s="8"/>
       <c r="E4" s="8"/>
       <c r="G4" s="8"/>
@@ -1570,11 +2494,68 @@
       <c r="W4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="X4" s="9" t="s">
-        <v>15</v>
+      <c r="Y4" t="s">
+        <v>21</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>25</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>27</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>29</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>30</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>31</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>32</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>33</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AQ4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AT4" t="s">
+        <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:46">
       <c r="C5" s="10"/>
       <c r="E5" s="10"/>
       <c r="G5" s="10"/>
@@ -1582,7 +2563,7 @@
       <c r="K5" s="10"/>
       <c r="M5" s="10"/>
       <c r="P5" s="11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="12"/>
       <c r="R5" s="13"/>
@@ -1591,11 +2572,90 @@
       <c r="U5" s="13"/>
       <c r="V5" s="13"/>
       <c r="W5" s="13"/>
-      <c r="X5" s="11"/>
+      <c r="Y5">
+        <f>IF(S5="",NA(),IF(S5=0,0.1,S5))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z5">
+        <f>IF(T5="",NA(),IF(T5=0,0.1,T5))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA5">
+        <f>IF(U5="",NA(),IF(U5=0,0.1,U5))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB5">
+        <f>IF(V5="",NA(),IF(V5=0,0.1,V5))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC5">
+        <f>IF(W5="",NA(),IF(W5=0,0.1,W5))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF5">
+        <f>IF(S5="",NA(),1+IF(AND(ABS(S5)&lt;=1,S5&gt;=0),-0.1,0))</f>
+        <v>0.9</v>
+      </c>
+      <c r="AG5">
+        <f>IF(S5="",NA(),IF(Y5&gt;=0,0+Y5/2,0+Y5/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH5" t="str">
+        <f>IF(S5="","",ROUND(S5,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI5">
+        <f>IF(T5="",NA(),1+IF(AND(ABS(T5)&lt;=1,T5&gt;=0),0.1,0))</f>
+        <v>1.1</v>
+      </c>
+      <c r="AJ5">
+        <f>IF(T5="",NA(),IF(Z5&gt;=0,SUMIF(Y5:Y5,"&gt;0",Y5:Y5)+Z5/2,SUMIF(Y5:Y5,"&lt;0",Y5:Y5)+Z5/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK5" t="str">
+        <f>IF(T5="","",ROUND(T5,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL5">
+        <f>IF(U5="",NA(),1+IF(AND(ABS(U5)&lt;=1,U5&gt;=0),0,0))</f>
+        <v>1</v>
+      </c>
+      <c r="AM5">
+        <f>IF(U5="",NA(),IF(AA5&gt;=0,SUMIF(Y5:Z5,"&gt;0",Y5:Z5)+AA5/2,SUMIF(Y5:Z5,"&lt;0",Y5:Z5)+AA5/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN5" t="str">
+        <f>IF(U5="","",ROUND(U5,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO5">
+        <f>IF(V5="",NA(),1+IF(AND(ABS(V5)&lt;=1,V5&gt;=0),0.08,0))</f>
+        <v>1.08</v>
+      </c>
+      <c r="AP5">
+        <f>IF(V5="",NA(),IF(AB5&gt;=0,SUMIF(Y5:AA5,"&gt;0",Y5:AA5)+AB5/2,SUMIF(Y5:AA5,"&lt;0",Y5:AA5)+AB5/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ5" t="str">
+        <f>IF(V5="","",ROUND(V5,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR5">
+        <f>IF(W5="",NA(),1+IF(AND(ABS(W5)&lt;=1,W5&gt;=0),-0.08,0))</f>
+        <v>0.92</v>
+      </c>
+      <c r="AS5">
+        <f>IF(W5="",NA(),IF(AC5&gt;=0,SUMIF(Y5:AB5,"&gt;0",Y5:AB5)+AC5/2,SUMIF(Y5:AB5,"&lt;0",Y5:AB5)+AC5/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT5" t="str">
+        <f>IF(W5="","",ROUND(W5,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
     </row>
-    <row r="6" spans="1:25">
+    <row r="6" spans="1:46">
       <c r="P6" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q6" s="12"/>
       <c r="R6" s="13"/>
@@ -1604,11 +2664,90 @@
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
       <c r="W6" s="13"/>
-      <c r="X6" s="11"/>
+      <c r="Y6">
+        <f>IF(S6="",NA(),IF(S6=0,0.1,S6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z6">
+        <f>IF(T6="",NA(),IF(T6=0,0.1,T6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA6">
+        <f>IF(U6="",NA(),IF(U6=0,0.1,U6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB6">
+        <f>IF(V6="",NA(),IF(V6=0,0.1,V6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC6">
+        <f>IF(W6="",NA(),IF(W6=0,0.1,W6))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF6">
+        <f>IF(S6="",NA(),2+IF(AND(ABS(S6)&lt;=1,S6&gt;=0),-0.1,0))</f>
+        <v>1.9</v>
+      </c>
+      <c r="AG6">
+        <f>IF(S6="",NA(),IF(Y6&gt;=0,0+Y6/2,0+Y6/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH6" t="str">
+        <f>IF(S6="","",ROUND(S6,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI6">
+        <f>IF(T6="",NA(),2+IF(AND(ABS(T6)&lt;=1,T6&gt;=0),0.1,0))</f>
+        <v>2.1</v>
+      </c>
+      <c r="AJ6">
+        <f>IF(T6="",NA(),IF(Z6&gt;=0,SUMIF(Y6:Y6,"&gt;0",Y6:Y6)+Z6/2,SUMIF(Y6:Y6,"&lt;0",Y6:Y6)+Z6/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK6" t="str">
+        <f>IF(T6="","",ROUND(T6,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL6">
+        <f>IF(U6="",NA(),2+IF(AND(ABS(U6)&lt;=1,U6&gt;=0),0,0))</f>
+        <v>2</v>
+      </c>
+      <c r="AM6">
+        <f>IF(U6="",NA(),IF(AA6&gt;=0,SUMIF(Y6:Z6,"&gt;0",Y6:Z6)+AA6/2,SUMIF(Y6:Z6,"&lt;0",Y6:Z6)+AA6/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN6" t="str">
+        <f>IF(U6="","",ROUND(U6,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO6">
+        <f>IF(V6="",NA(),2+IF(AND(ABS(V6)&lt;=1,V6&gt;=0),0.08,0))</f>
+        <v>2.08</v>
+      </c>
+      <c r="AP6">
+        <f>IF(V6="",NA(),IF(AB6&gt;=0,SUMIF(Y6:AA6,"&gt;0",Y6:AA6)+AB6/2,SUMIF(Y6:AA6,"&lt;0",Y6:AA6)+AB6/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ6" t="str">
+        <f>IF(V6="","",ROUND(V6,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR6">
+        <f>IF(W6="",NA(),2+IF(AND(ABS(W6)&lt;=1,W6&gt;=0),-0.08,0))</f>
+        <v>1.92</v>
+      </c>
+      <c r="AS6">
+        <f>IF(W6="",NA(),IF(AC6&gt;=0,SUMIF(Y6:AB6,"&gt;0",Y6:AB6)+AC6/2,SUMIF(Y6:AB6,"&lt;0",Y6:AB6)+AC6/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT6" t="str">
+        <f>IF(W6="","",ROUND(W6,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:46">
       <c r="P7" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Q7" s="12"/>
       <c r="R7" s="13"/>
@@ -1617,11 +2756,90 @@
       <c r="U7" s="13"/>
       <c r="V7" s="13"/>
       <c r="W7" s="13"/>
-      <c r="X7" s="11"/>
+      <c r="Y7">
+        <f>IF(S7="",NA(),IF(S7=0,0.1,S7))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z7">
+        <f>IF(T7="",NA(),IF(T7=0,0.1,T7))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA7">
+        <f>IF(U7="",NA(),IF(U7=0,0.1,U7))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB7">
+        <f>IF(V7="",NA(),IF(V7=0,0.1,V7))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC7">
+        <f>IF(W7="",NA(),IF(W7=0,0.1,W7))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF7">
+        <f>IF(S7="",NA(),3+IF(AND(ABS(S7)&lt;=1,S7&gt;=0),-0.1,0))</f>
+        <v>2.9</v>
+      </c>
+      <c r="AG7">
+        <f>IF(S7="",NA(),IF(Y7&gt;=0,0+Y7/2,0+Y7/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH7" t="str">
+        <f>IF(S7="","",ROUND(S7,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI7">
+        <f>IF(T7="",NA(),3+IF(AND(ABS(T7)&lt;=1,T7&gt;=0),0.1,0))</f>
+        <v>3.1</v>
+      </c>
+      <c r="AJ7">
+        <f>IF(T7="",NA(),IF(Z7&gt;=0,SUMIF(Y7:Y7,"&gt;0",Y7:Y7)+Z7/2,SUMIF(Y7:Y7,"&lt;0",Y7:Y7)+Z7/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK7" t="str">
+        <f>IF(T7="","",ROUND(T7,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL7">
+        <f>IF(U7="",NA(),3+IF(AND(ABS(U7)&lt;=1,U7&gt;=0),0,0))</f>
+        <v>3</v>
+      </c>
+      <c r="AM7">
+        <f>IF(U7="",NA(),IF(AA7&gt;=0,SUMIF(Y7:Z7,"&gt;0",Y7:Z7)+AA7/2,SUMIF(Y7:Z7,"&lt;0",Y7:Z7)+AA7/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN7" t="str">
+        <f>IF(U7="","",ROUND(U7,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO7">
+        <f>IF(V7="",NA(),3+IF(AND(ABS(V7)&lt;=1,V7&gt;=0),0.08,0))</f>
+        <v>3.08</v>
+      </c>
+      <c r="AP7">
+        <f>IF(V7="",NA(),IF(AB7&gt;=0,SUMIF(Y7:AA7,"&gt;0",Y7:AA7)+AB7/2,SUMIF(Y7:AA7,"&lt;0",Y7:AA7)+AB7/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ7" t="str">
+        <f>IF(V7="","",ROUND(V7,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR7">
+        <f>IF(W7="",NA(),3+IF(AND(ABS(W7)&lt;=1,W7&gt;=0),-0.08,0))</f>
+        <v>2.92</v>
+      </c>
+      <c r="AS7">
+        <f>IF(W7="",NA(),IF(AC7&gt;=0,SUMIF(Y7:AB7,"&gt;0",Y7:AB7)+AC7/2,SUMIF(Y7:AB7,"&lt;0",Y7:AB7)+AC7/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT7" t="str">
+        <f>IF(W7="","",ROUND(W7,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:46">
       <c r="P8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="Q8" s="12"/>
       <c r="R8" s="13"/>
@@ -1630,11 +2848,90 @@
       <c r="U8" s="13"/>
       <c r="V8" s="13"/>
       <c r="W8" s="13"/>
-      <c r="X8" s="11"/>
+      <c r="Y8">
+        <f>IF(S8="",NA(),IF(S8=0,0.1,S8))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z8">
+        <f>IF(T8="",NA(),IF(T8=0,0.1,T8))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA8">
+        <f>IF(U8="",NA(),IF(U8=0,0.1,U8))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB8">
+        <f>IF(V8="",NA(),IF(V8=0,0.1,V8))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC8">
+        <f>IF(W8="",NA(),IF(W8=0,0.1,W8))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF8">
+        <f>IF(S8="",NA(),4+IF(AND(ABS(S8)&lt;=1,S8&gt;=0),-0.1,0))</f>
+        <v>3.9</v>
+      </c>
+      <c r="AG8">
+        <f>IF(S8="",NA(),IF(Y8&gt;=0,0+Y8/2,0+Y8/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH8" t="str">
+        <f>IF(S8="","",ROUND(S8,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI8">
+        <f>IF(T8="",NA(),4+IF(AND(ABS(T8)&lt;=1,T8&gt;=0),0.1,0))</f>
+        <v>4.1</v>
+      </c>
+      <c r="AJ8">
+        <f>IF(T8="",NA(),IF(Z8&gt;=0,SUMIF(Y8:Y8,"&gt;0",Y8:Y8)+Z8/2,SUMIF(Y8:Y8,"&lt;0",Y8:Y8)+Z8/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK8" t="str">
+        <f>IF(T8="","",ROUND(T8,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL8">
+        <f>IF(U8="",NA(),4+IF(AND(ABS(U8)&lt;=1,U8&gt;=0),0,0))</f>
+        <v>4</v>
+      </c>
+      <c r="AM8">
+        <f>IF(U8="",NA(),IF(AA8&gt;=0,SUMIF(Y8:Z8,"&gt;0",Y8:Z8)+AA8/2,SUMIF(Y8:Z8,"&lt;0",Y8:Z8)+AA8/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN8" t="str">
+        <f>IF(U8="","",ROUND(U8,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO8">
+        <f>IF(V8="",NA(),4+IF(AND(ABS(V8)&lt;=1,V8&gt;=0),0.08,0))</f>
+        <v>4.08</v>
+      </c>
+      <c r="AP8">
+        <f>IF(V8="",NA(),IF(AB8&gt;=0,SUMIF(Y8:AA8,"&gt;0",Y8:AA8)+AB8/2,SUMIF(Y8:AA8,"&lt;0",Y8:AA8)+AB8/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ8" t="str">
+        <f>IF(V8="","",ROUND(V8,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR8">
+        <f>IF(W8="",NA(),4+IF(AND(ABS(W8)&lt;=1,W8&gt;=0),-0.08,0))</f>
+        <v>3.92</v>
+      </c>
+      <c r="AS8">
+        <f>IF(W8="",NA(),IF(AC8&gt;=0,SUMIF(Y8:AB8,"&gt;0",Y8:AB8)+AC8/2,SUMIF(Y8:AB8,"&lt;0",Y8:AB8)+AC8/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT8" t="str">
+        <f>IF(W8="","",ROUND(W8,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:46">
       <c r="P9" s="11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="Q9" s="12"/>
       <c r="R9" s="13"/>
@@ -1643,13 +2940,90 @@
       <c r="U9" s="13"/>
       <c r="V9" s="13"/>
       <c r="W9" s="13"/>
-      <c r="X9" s="11" t="s">
-        <v>21</v>
+      <c r="Y9">
+        <f>IF(S9="",NA(),IF(S9=0,0.1,S9))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z9">
+        <f>IF(T9="",NA(),IF(T9=0,0.1,T9))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA9">
+        <f>IF(U9="",NA(),IF(U9=0,0.1,U9))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB9">
+        <f>IF(V9="",NA(),IF(V9=0,0.1,V9))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC9">
+        <f>IF(W9="",NA(),IF(W9=0,0.1,W9))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF9">
+        <f>IF(S9="",NA(),5+IF(AND(ABS(S9)&lt;=1,S9&gt;=0),-0.1,0))</f>
+        <v>4.9</v>
+      </c>
+      <c r="AG9">
+        <f>IF(S9="",NA(),IF(Y9&gt;=0,0+Y9/2,0+Y9/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH9" t="str">
+        <f>IF(S9="","",ROUND(S9,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI9">
+        <f>IF(T9="",NA(),5+IF(AND(ABS(T9)&lt;=1,T9&gt;=0),0.1,0))</f>
+        <v>5.1</v>
+      </c>
+      <c r="AJ9">
+        <f>IF(T9="",NA(),IF(Z9&gt;=0,SUMIF(Y9:Y9,"&gt;0",Y9:Y9)+Z9/2,SUMIF(Y9:Y9,"&lt;0",Y9:Y9)+Z9/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK9" t="str">
+        <f>IF(T9="","",ROUND(T9,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL9">
+        <f>IF(U9="",NA(),5+IF(AND(ABS(U9)&lt;=1,U9&gt;=0),0,0))</f>
+        <v>5</v>
+      </c>
+      <c r="AM9">
+        <f>IF(U9="",NA(),IF(AA9&gt;=0,SUMIF(Y9:Z9,"&gt;0",Y9:Z9)+AA9/2,SUMIF(Y9:Z9,"&lt;0",Y9:Z9)+AA9/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN9" t="str">
+        <f>IF(U9="","",ROUND(U9,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO9">
+        <f>IF(V9="",NA(),5+IF(AND(ABS(V9)&lt;=1,V9&gt;=0),0.08,0))</f>
+        <v>5.08</v>
+      </c>
+      <c r="AP9">
+        <f>IF(V9="",NA(),IF(AB9&gt;=0,SUMIF(Y9:AA9,"&gt;0",Y9:AA9)+AB9/2,SUMIF(Y9:AA9,"&lt;0",Y9:AA9)+AB9/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ9" t="str">
+        <f>IF(V9="","",ROUND(V9,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR9">
+        <f>IF(W9="",NA(),5+IF(AND(ABS(W9)&lt;=1,W9&gt;=0),-0.08,0))</f>
+        <v>4.92</v>
+      </c>
+      <c r="AS9">
+        <f>IF(W9="",NA(),IF(AC9&gt;=0,SUMIF(Y9:AB9,"&gt;0",Y9:AB9)+AC9/2,SUMIF(Y9:AB9,"&lt;0",Y9:AB9)+AC9/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT9" t="str">
+        <f>IF(W9="","",ROUND(W9,0)&amp;"%")</f>
+        <v>0%</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:46">
       <c r="P10" s="11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="Q10" s="12"/>
       <c r="R10" s="13"/>
@@ -1658,16 +3032,93 @@
       <c r="U10" s="13"/>
       <c r="V10" s="13"/>
       <c r="W10" s="13"/>
-      <c r="X10" s="11" t="s">
-        <v>21</v>
+      <c r="Y10">
+        <f>IF(S10="",NA(),IF(S10=0,0.1,S10))</f>
+        <v>0.1</v>
+      </c>
+      <c r="Z10">
+        <f>IF(T10="",NA(),IF(T10=0,0.1,T10))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AA10">
+        <f>IF(U10="",NA(),IF(U10=0,0.1,U10))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AB10">
+        <f>IF(V10="",NA(),IF(V10=0,0.1,V10))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AC10">
+        <f>IF(W10="",NA(),IF(W10=0,0.1,W10))</f>
+        <v>0.1</v>
+      </c>
+      <c r="AF10">
+        <f>IF(S10="",NA(),6+IF(AND(ABS(S10)&lt;=1,S10&gt;=0),-0.1,0))</f>
+        <v>5.9</v>
+      </c>
+      <c r="AG10">
+        <f>IF(S10="",NA(),IF(Y10&gt;=0,0+Y10/2,0+Y10/2))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AH10" t="str">
+        <f>IF(S10="","",ROUND(S10,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AI10">
+        <f>IF(T10="",NA(),6+IF(AND(ABS(T10)&lt;=1,T10&gt;=0),0.1,0))</f>
+        <v>6.1</v>
+      </c>
+      <c r="AJ10">
+        <f>IF(T10="",NA(),IF(Z10&gt;=0,SUMIF(Y10:Y10,"&gt;0",Y10:Y10)+Z10/2,SUMIF(Y10:Y10,"&lt;0",Y10:Y10)+Z10/2))</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="AK10" t="str">
+        <f>IF(T10="","",ROUND(T10,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AL10">
+        <f>IF(U10="",NA(),6+IF(AND(ABS(U10)&lt;=1,U10&gt;=0),0,0))</f>
+        <v>6</v>
+      </c>
+      <c r="AM10">
+        <f>IF(U10="",NA(),IF(AA10&gt;=0,SUMIF(Y10:Z10,"&gt;0",Y10:Z10)+AA10/2,SUMIF(Y10:Z10,"&lt;0",Y10:Z10)+AA10/2))</f>
+        <v>0.25</v>
+      </c>
+      <c r="AN10" t="str">
+        <f>IF(U10="","",ROUND(U10,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AO10">
+        <f>IF(V10="",NA(),6+IF(AND(ABS(V10)&lt;=1,V10&gt;=0),0.08,0))</f>
+        <v>6.08</v>
+      </c>
+      <c r="AP10">
+        <f>IF(V10="",NA(),IF(AB10&gt;=0,SUMIF(Y10:AA10,"&gt;0",Y10:AA10)+AB10/2,SUMIF(Y10:AA10,"&lt;0",Y10:AA10)+AB10/2))</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="AQ10" t="str">
+        <f>IF(V10="","",ROUND(V10,0)&amp;"%")</f>
+        <v>0%</v>
+      </c>
+      <c r="AR10">
+        <f>IF(W10="",NA(),6+IF(AND(ABS(W10)&lt;=1,W10&gt;=0),-0.08,0))</f>
+        <v>5.92</v>
+      </c>
+      <c r="AS10">
+        <f>IF(W10="",NA(),IF(AC10&gt;=0,SUMIF(Y10:AB10,"&gt;0",Y10:AB10)+AC10/2,SUMIF(Y10:AB10,"&lt;0",Y10:AB10)+AC10/2))</f>
+        <v>0.45</v>
+      </c>
+      <c r="AT10" t="str">
+        <f>IF(W10="","",ROUND(W10,0)&amp;"%")</f>
+        <v>0%</v>
       </c>
     </row>
-    <row r="11" spans="1:25"/>
-    <row r="12" spans="1:25"/>
-    <row r="13" spans="1:25"/>
-    <row r="14" spans="1:25"/>
-    <row r="15" spans="1:25"/>
-    <row r="16" spans="1:25"/>
+    <row r="11" spans="1:46"/>
+    <row r="12" spans="1:46"/>
+    <row r="13" spans="1:46"/>
+    <row r="14" spans="1:46"/>
+    <row r="15" spans="1:46"/>
+    <row r="16" spans="1:46"/>
     <row r="17"/>
     <row r="18"/>
     <row r="19"/>
@@ -1697,14 +3148,4 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>